<commit_message>
Rework Sucre app as full Grill clone plus people-only actors
Replace the stripped-down Sucre mini-app with the complete Grill
xlsx pipeline (normalization, duplicates, tono/tema/subtema, PKL,
Link style, Sheets) and append four actor columns. Propios and
externos accept only named people; Lucy is omitted unless she
intervenes; extracts stay verbatim from CuerpoEs.

Co-authored-by: johnathanacortesd <johnathanacortesd@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/sucre_dossier_ejemplo.xlsx
+++ b/samples/sucre_dossier_ejemplo.xlsx
@@ -425,13 +425,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>NoticiaId</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -441,17 +441,47 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo de Medio</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Título</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>CuerpoEs</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>URL Nota</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Empresa rel.</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>URL Nota AV</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Menciones - Empresa</t>
         </is>
       </c>
     </row>
@@ -466,19 +496,41 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>El Meridiano</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Gobernadora Lucy García entregó 200 becas en Sincelejo</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>La gobernadora Lucy García Montes entregó 200 becas universitarias en Sincelejo. "La educación es la prioridad de este gobierno", afirmó la mandataria. El alcalde Ricardo Hernández felicitó a la gobernadora por la inversión social.</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://example.com/becas</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Gobernación de Sucre</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -491,19 +543,41 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>El Heraldo</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Senador cuestiona ejecución de vías en Sucre</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>El senador Andrés Pérez señaló que la Gobernación de Sucre no ha ejecutado el presupuesto de vías rurales y pidió explicaciones a la mandataria.</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://example.com/vias</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Gobernación de Sucre</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -516,17 +590,39 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>RCN Radio</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Secretaría de Educación departamental expide resolución de cobertura</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>La Secretaría de Educación departamental emitió la Resolución 045 de 2026 para ampliar la cobertura escolar en los municipios del Golfo de Morrosquillo.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://example.com/resolucion</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Gobernación de Sucre</t>
         </is>
       </c>
     </row>
@@ -541,19 +637,182 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>11:00:00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Caracol</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Boletín climático del Ideam para la región Caribe</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>El Ideam publicó el pronóstico de lluvias para la región Caribe. No se registran declaraciones de autoridades departamentales de Sucre.</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://example.com/clima</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Ideam</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>El Universal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Secretario de Educación de Sucre anuncia ampliación de cupos</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>El secretario de Educación de Sucre, Carlos Méndez, anunció la ampliación de cupos escolares en Sincelejo y reiteró el compromiso de la Gobernación.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://example.com/cupos</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Gobernación de Sucre</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>13:00:00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>La República</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Gobernación de Sucre emite comunicado presupuestal</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>La Gobernación de Sucre emitió un comunicado sobre el presupuesto de 2026 sin declaraciones de la mandataria ni de secretarios.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://example.com/presupuesto</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Gobernación de Sucre</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>El Colombiano</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Gobernador de Antioquia se refiere a la gestión en Sucre</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Andrés Julián Rendón, Gobernador de Antioquia, afirmó que la Gobernación de Sucre puede replicar el modelo de vías terciarias del occidente antioqueño.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://example.com/rendon</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Gobernación de Sucre</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>